<commit_message>
Primer registro de decision
</commit_message>
<xml_diff>
--- a/Registro de decisiones.xlsx
+++ b/Registro de decisiones.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bdf77c9882a5fb43/Escritorio/laboratorio/novamarket-checkout-service/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="5" documentId="8_{F87E22D3-17D3-41A7-98E0-7C8DA0BE2010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{A4119A81-A85F-4E2C-A647-7209E9B2B521}"/>
+  <xr:revisionPtr revIDLastSave="27" documentId="8_{F87E22D3-17D3-41A7-98E0-7C8DA0BE2010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F22FB97C-D276-4AF3-A50C-0B10FA843C9D}"/>
   <bookViews>
-    <workbookView xWindow="11424" yWindow="0" windowWidth="11712" windowHeight="12336" xr2:uid="{C6AF2156-5091-4E8F-AD24-4F68CDB55078}"/>
+    <workbookView xWindow="6072" yWindow="1392" windowWidth="17280" windowHeight="8964" xr2:uid="{C6AF2156-5091-4E8F-AD24-4F68CDB55078}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
   <si>
     <t>ID</t>
   </si>
@@ -57,6 +57,18 @@
   </si>
   <si>
     <t>Registro de decisiones</t>
+  </si>
+  <si>
+    <t>Crear rama NM-101 en local</t>
+  </si>
+  <si>
+    <t>En local podemos editar sin riesgo de afectar al principal remoto</t>
+  </si>
+  <si>
+    <t>Crear rama desde remoto</t>
+  </si>
+  <si>
+    <t>Riesgo de una mala decisión y quede registrado en el historial</t>
   </si>
 </sst>
 </file>
@@ -88,7 +100,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="3">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -120,16 +132,54 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="8">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -146,6 +196,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -468,9 +522,10 @@
   <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="3" max="3" width="18.33203125" customWidth="1"/>
+    <col min="2" max="2" width="25.5546875" customWidth="1"/>
+    <col min="3" max="3" width="44" customWidth="1"/>
     <col min="4" max="4" width="29.44140625" customWidth="1"/>
-    <col min="5" max="5" width="19.109375" customWidth="1"/>
+    <col min="5" max="5" width="32.5546875" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
@@ -500,18 +555,28 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="2"/>
-      <c r="B3" s="2"/>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
+      <c r="A3" s="4">
+        <v>1</v>
+      </c>
+      <c r="B3" s="6" t="s">
+        <v>6</v>
+      </c>
+      <c r="C3" s="6" t="s">
+        <v>7</v>
+      </c>
+      <c r="D3" s="6" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" s="6" t="s">
+        <v>9</v>
+      </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="2"/>
-      <c r="B4" s="2"/>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
+      <c r="A4" s="5"/>
+      <c r="B4" s="7"/>
+      <c r="C4" s="7"/>
+      <c r="D4" s="7"/>
+      <c r="E4" s="7"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="2"/>
@@ -612,8 +677,13 @@
       <c r="E18" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="6">
     <mergeCell ref="A1:E1"/>
+    <mergeCell ref="C3:C4"/>
+    <mergeCell ref="A3:A4"/>
+    <mergeCell ref="B3:B4"/>
+    <mergeCell ref="D3:D4"/>
+    <mergeCell ref="E3:E4"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Segundo registro de decision
</commit_message>
<xml_diff>
--- a/Registro de decisiones.xlsx
+++ b/Registro de decisiones.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bdf77c9882a5fb43/Escritorio/laboratorio/novamarket-checkout-service/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="27" documentId="8_{F87E22D3-17D3-41A7-98E0-7C8DA0BE2010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F22FB97C-D276-4AF3-A50C-0B10FA843C9D}"/>
+  <xr:revisionPtr revIDLastSave="42" documentId="8_{F87E22D3-17D3-41A7-98E0-7C8DA0BE2010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37C8CC4F-697F-4870-B504-F3CEEA7D388E}"/>
   <bookViews>
-    <workbookView xWindow="6072" yWindow="1392" windowWidth="17280" windowHeight="8964" xr2:uid="{C6AF2156-5091-4E8F-AD24-4F68CDB55078}"/>
+    <workbookView xWindow="4212" yWindow="1908" windowWidth="17280" windowHeight="8964" xr2:uid="{C6AF2156-5091-4E8F-AD24-4F68CDB55078}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
   <si>
     <t>ID</t>
   </si>
@@ -69,6 +69,18 @@
   </si>
   <si>
     <t>Riesgo de una mala decisión y quede registrado en el historial</t>
+  </si>
+  <si>
+    <t>Revisión de rama NM -101 en remoto</t>
+  </si>
+  <si>
+    <t>Ampliar la validación de entornos del archivo intalacion creando el proceso NM-102</t>
+  </si>
+  <si>
+    <t>Crear rama para proceso NM-102</t>
+  </si>
+  <si>
+    <t>No sabría en que rama de configuración se está trabajando</t>
   </si>
 </sst>
 </file>
@@ -170,16 +182,16 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -555,84 +567,94 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="4">
+      <c r="A3" s="6">
         <v>1</v>
       </c>
-      <c r="B3" s="6" t="s">
+      <c r="B3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="6" t="s">
+      <c r="C3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="6" t="s">
+      <c r="D3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="6" t="s">
+      <c r="E3" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="5"/>
-      <c r="B4" s="7"/>
-      <c r="C4" s="7"/>
-      <c r="D4" s="7"/>
-      <c r="E4" s="7"/>
+      <c r="A4" s="7"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="2"/>
-      <c r="B5" s="2"/>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
+      <c r="A5" s="6">
+        <v>2</v>
+      </c>
+      <c r="B5" s="4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C5" s="4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" s="4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" s="4" t="s">
+        <v>13</v>
+      </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="2"/>
-      <c r="B6" s="2"/>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
+      <c r="A6" s="7"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="2"/>
-      <c r="B7" s="2"/>
-      <c r="C7" s="2"/>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
+      <c r="A7" s="6"/>
+      <c r="B7" s="4"/>
+      <c r="C7" s="4"/>
+      <c r="D7" s="4"/>
+      <c r="E7" s="4"/>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="2"/>
-      <c r="B8" s="2"/>
-      <c r="C8" s="2"/>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
+      <c r="A8" s="7"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
+      <c r="A9" s="6"/>
+      <c r="B9" s="4"/>
+      <c r="C9" s="4"/>
+      <c r="D9" s="4"/>
+      <c r="E9" s="4"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="2"/>
-      <c r="B10" s="2"/>
-      <c r="C10" s="2"/>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
+      <c r="A10" s="7"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="2"/>
-      <c r="B11" s="2"/>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="2"/>
-      <c r="B12" s="2"/>
-      <c r="C12" s="2"/>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
+      <c r="A12" s="7"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
@@ -677,7 +699,27 @@
       <c r="E18" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="26">
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="A3:A4"/>

</xml_diff>

<commit_message>
Tercer registro de decision
</commit_message>
<xml_diff>
--- a/Registro de decisiones.xlsx
+++ b/Registro de decisiones.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bdf77c9882a5fb43/Escritorio/laboratorio/novamarket-checkout-service/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="42" documentId="8_{F87E22D3-17D3-41A7-98E0-7C8DA0BE2010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{37C8CC4F-697F-4870-B504-F3CEEA7D388E}"/>
+  <xr:revisionPtr revIDLastSave="51" documentId="8_{F87E22D3-17D3-41A7-98E0-7C8DA0BE2010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40883E3E-31C9-4E34-B01C-05C4A2629077}"/>
   <bookViews>
-    <workbookView xWindow="4212" yWindow="1908" windowWidth="17280" windowHeight="8964" xr2:uid="{C6AF2156-5091-4E8F-AD24-4F68CDB55078}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C6AF2156-5091-4E8F-AD24-4F68CDB55078}"/>
   </bookViews>
   <sheets>
     <sheet name="Hoja1" sheetId="1" r:id="rId1"/>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="14">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>ID</t>
   </si>
@@ -81,6 +81,18 @@
   </si>
   <si>
     <t>No sabría en que rama de configuración se está trabajando</t>
+  </si>
+  <si>
+    <t>Crear archivo validacion-entornos en local</t>
+  </si>
+  <si>
+    <t>Los que tienen vinculo con el proyecto no pueden ver las actualizaciones hasta enviar a remoto</t>
+  </si>
+  <si>
+    <t>Crear archivo validacion-entornos en remoto</t>
+  </si>
+  <si>
+    <t>Los usuarios pueden ver las validaciones en tiempo real y pueden actualizar el archivo hasta complicar el proceso</t>
   </si>
 </sst>
 </file>
@@ -178,7 +190,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -187,10 +202,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -537,17 +549,17 @@
     <col min="2" max="2" width="25.5546875" customWidth="1"/>
     <col min="3" max="3" width="44" customWidth="1"/>
     <col min="4" max="4" width="29.44140625" customWidth="1"/>
-    <col min="5" max="5" width="32.5546875" customWidth="1"/>
+    <col min="5" max="5" width="47.109375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -567,94 +579,104 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="6">
+      <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="7"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
+      <c r="A4" s="4"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="6">
+      <c r="A5" s="3">
         <v>2</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="7"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
+      <c r="A6" s="4"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="6"/>
-      <c r="B7" s="4"/>
-      <c r="C7" s="4"/>
-      <c r="D7" s="4"/>
-      <c r="E7" s="4"/>
+      <c r="A7" s="3">
+        <v>3</v>
+      </c>
+      <c r="B7" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="C7" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="D7" s="5" t="s">
+        <v>16</v>
+      </c>
+      <c r="E7" s="5" t="s">
+        <v>17</v>
+      </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="7"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
+      <c r="A8" s="4"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="6"/>
-      <c r="B9" s="4"/>
-      <c r="C9" s="4"/>
-      <c r="D9" s="4"/>
-      <c r="E9" s="4"/>
+      <c r="A9" s="3"/>
+      <c r="B9" s="5"/>
+      <c r="C9" s="5"/>
+      <c r="D9" s="5"/>
+      <c r="E9" s="5"/>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="7"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
+      <c r="A10" s="4"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="6"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
+      <c r="A11" s="3"/>
+      <c r="B11" s="5"/>
+      <c r="C11" s="5"/>
+      <c r="D11" s="5"/>
+      <c r="E11" s="5"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="7"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
+      <c r="A12" s="4"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
@@ -700,32 +722,32 @@
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="E3:E4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Cuarto registro de decision
</commit_message>
<xml_diff>
--- a/Registro de decisiones.xlsx
+++ b/Registro de decisiones.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bdf77c9882a5fb43/Escritorio/laboratorio/novamarket-checkout-service/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bdf77c9882a5fb43/Escritorio/laboratorio/fork1-novamarket-checkout-service/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="51" documentId="8_{F87E22D3-17D3-41A7-98E0-7C8DA0BE2010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{40883E3E-31C9-4E34-B01C-05C4A2629077}"/>
+  <xr:revisionPtr revIDLastSave="58" documentId="8_{F87E22D3-17D3-41A7-98E0-7C8DA0BE2010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30075D1F-AB21-4921-860F-8630F9F278EF}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C6AF2156-5091-4E8F-AD24-4F68CDB55078}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
   <si>
     <t>ID</t>
   </si>
@@ -93,6 +93,18 @@
   </si>
   <si>
     <t>Los usuarios pueden ver las validaciones en tiempo real y pueden actualizar el archivo hasta complicar el proceso</t>
+  </si>
+  <si>
+    <t>Creación de Fork en remoto</t>
+  </si>
+  <si>
+    <t>Copia todos los archivos del respositorio principal</t>
+  </si>
+  <si>
+    <t>Dar permisos al repositorio principal</t>
+  </si>
+  <si>
+    <t>Otorgar permisos a personas externas compromete el servicio principal por una mala gestión</t>
   </si>
 </sst>
 </file>
@@ -190,10 +202,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -202,7 +211,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -220,10 +232,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -553,13 +561,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -579,104 +587,114 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="3">
+      <c r="A3" s="6">
         <v>1</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="4"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
+      <c r="A4" s="7"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="3">
+      <c r="A5" s="6">
         <v>2</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="4" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="4"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
+      <c r="A6" s="7"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="3">
+      <c r="A7" s="6">
         <v>3</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="4" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="4"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
+      <c r="A8" s="7"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="3"/>
-      <c r="B9" s="5"/>
-      <c r="C9" s="5"/>
-      <c r="D9" s="5"/>
-      <c r="E9" s="5"/>
+      <c r="A9" s="6">
+        <v>4</v>
+      </c>
+      <c r="B9" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="C9" s="4" t="s">
+        <v>19</v>
+      </c>
+      <c r="D9" s="4" t="s">
+        <v>20</v>
+      </c>
+      <c r="E9" s="4" t="s">
+        <v>21</v>
+      </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="4"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
+      <c r="A10" s="7"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="3"/>
-      <c r="B11" s="5"/>
-      <c r="C11" s="5"/>
-      <c r="D11" s="5"/>
-      <c r="E11" s="5"/>
+      <c r="A11" s="6"/>
+      <c r="B11" s="4"/>
+      <c r="C11" s="4"/>
+      <c r="D11" s="4"/>
+      <c r="E11" s="4"/>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="4"/>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
+      <c r="A12" s="7"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
@@ -722,32 +740,32 @@
     </row>
   </sheetData>
   <mergeCells count="26">
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="E3:E4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Quinta registro de decision
</commit_message>
<xml_diff>
--- a/Registro de decisiones.xlsx
+++ b/Registro de decisiones.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bdf77c9882a5fb43/Escritorio/laboratorio/fork1-novamarket-checkout-service/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="58" documentId="8_{F87E22D3-17D3-41A7-98E0-7C8DA0BE2010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{30075D1F-AB21-4921-860F-8630F9F278EF}"/>
+  <xr:revisionPtr revIDLastSave="63" documentId="8_{F87E22D3-17D3-41A7-98E0-7C8DA0BE2010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A0E499A-FFF1-4B06-AAFF-31A9385C4FBA}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C6AF2156-5091-4E8F-AD24-4F68CDB55078}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="22" uniqueCount="22">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
   <si>
     <t>ID</t>
   </si>
@@ -105,6 +105,18 @@
   </si>
   <si>
     <t>Otorgar permisos a personas externas compromete el servicio principal por una mala gestión</t>
+  </si>
+  <si>
+    <t>Editar archivo README en rama NM-103 local</t>
+  </si>
+  <si>
+    <t>Permite realizar cambios sin afectar al repositorio remoto hasta tener una respuesta clara</t>
+  </si>
+  <si>
+    <t>Editar en rama remota</t>
+  </si>
+  <si>
+    <t>Puede generar confusiones de actualizaciones al personal interno que desea revisar las propuestas externas</t>
   </si>
 </sst>
 </file>
@@ -202,7 +214,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -211,10 +226,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -232,6 +244,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -561,13 +577,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -587,114 +603,124 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="6">
+      <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="7"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
+      <c r="A4" s="4"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="6">
+      <c r="A5" s="3">
         <v>2</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="7"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
+      <c r="A6" s="4"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="6">
+      <c r="A7" s="3">
         <v>3</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="5" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="7"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
+      <c r="A8" s="4"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="6">
+      <c r="A9" s="3">
         <v>4</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="5" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="7"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
+      <c r="A10" s="4"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="6"/>
-      <c r="B11" s="4"/>
-      <c r="C11" s="4"/>
-      <c r="D11" s="4"/>
-      <c r="E11" s="4"/>
+      <c r="A11" s="3">
+        <v>5</v>
+      </c>
+      <c r="B11" s="5" t="s">
+        <v>22</v>
+      </c>
+      <c r="C11" s="5" t="s">
+        <v>23</v>
+      </c>
+      <c r="D11" s="5" t="s">
+        <v>24</v>
+      </c>
+      <c r="E11" s="5" t="s">
+        <v>25</v>
+      </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="7"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
+      <c r="A12" s="4"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="2"/>
@@ -740,32 +766,32 @@
     </row>
   </sheetData>
   <mergeCells count="26">
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="E3:E4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Sexto registro de decision
</commit_message>
<xml_diff>
--- a/Registro de decisiones.xlsx
+++ b/Registro de decisiones.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bdf77c9882a5fb43/Escritorio/laboratorio/fork1-novamarket-checkout-service/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bdf77c9882a5fb43/Escritorio/laboratorio/novamarket-checkout-service/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="63" documentId="8_{F87E22D3-17D3-41A7-98E0-7C8DA0BE2010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{9A0E499A-FFF1-4B06-AAFF-31A9385C4FBA}"/>
+  <xr:revisionPtr revIDLastSave="73" documentId="8_{F87E22D3-17D3-41A7-98E0-7C8DA0BE2010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD5B3CDD-02AF-427A-A36C-AAF1B981B8EE}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C6AF2156-5091-4E8F-AD24-4F68CDB55078}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="26" uniqueCount="26">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
   <si>
     <t>ID</t>
   </si>
@@ -117,6 +117,18 @@
   </si>
   <si>
     <t>Puede generar confusiones de actualizaciones al personal interno que desea revisar las propuestas externas</t>
+  </si>
+  <si>
+    <t>Merge de repositorio fork al principal</t>
+  </si>
+  <si>
+    <t>Primero se validó el proyecto NM-103 y cumple con todos los parámetros establecidos</t>
+  </si>
+  <si>
+    <t>Realizar Merge sin validar</t>
+  </si>
+  <si>
+    <t>No validar que cambios se realizó puede poner en riesgo el proyecto principal</t>
   </si>
 </sst>
 </file>
@@ -214,10 +226,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -226,7 +235,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -244,10 +256,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
-<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -577,13 +585,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="7" t="s">
+      <c r="A1" s="3" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="7"/>
-      <c r="C1" s="7"/>
-      <c r="D1" s="7"/>
-      <c r="E1" s="7"/>
+      <c r="B1" s="3"/>
+      <c r="C1" s="3"/>
+      <c r="D1" s="3"/>
+      <c r="E1" s="3"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -603,152 +611,162 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="3">
+      <c r="A3" s="6">
         <v>1</v>
       </c>
-      <c r="B3" s="5" t="s">
+      <c r="B3" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="5" t="s">
+      <c r="C3" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="5" t="s">
+      <c r="D3" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="5" t="s">
+      <c r="E3" s="4" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="4"/>
-      <c r="B4" s="6"/>
-      <c r="C4" s="6"/>
-      <c r="D4" s="6"/>
-      <c r="E4" s="6"/>
+      <c r="A4" s="7"/>
+      <c r="B4" s="5"/>
+      <c r="C4" s="5"/>
+      <c r="D4" s="5"/>
+      <c r="E4" s="5"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="3">
+      <c r="A5" s="6">
         <v>2</v>
       </c>
-      <c r="B5" s="5" t="s">
+      <c r="B5" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="5" t="s">
+      <c r="C5" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="5" t="s">
+      <c r="D5" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="5" t="s">
+      <c r="E5" s="4" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="4"/>
-      <c r="B6" s="6"/>
-      <c r="C6" s="6"/>
-      <c r="D6" s="6"/>
-      <c r="E6" s="6"/>
+      <c r="A6" s="7"/>
+      <c r="B6" s="5"/>
+      <c r="C6" s="5"/>
+      <c r="D6" s="5"/>
+      <c r="E6" s="5"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="3">
+      <c r="A7" s="6">
         <v>3</v>
       </c>
-      <c r="B7" s="5" t="s">
+      <c r="B7" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="5" t="s">
+      <c r="C7" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="5" t="s">
+      <c r="D7" s="4" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="5" t="s">
+      <c r="E7" s="4" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="4"/>
-      <c r="B8" s="6"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
+      <c r="A8" s="7"/>
+      <c r="B8" s="5"/>
+      <c r="C8" s="5"/>
+      <c r="D8" s="5"/>
+      <c r="E8" s="5"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="3">
+      <c r="A9" s="6">
         <v>4</v>
       </c>
-      <c r="B9" s="5" t="s">
+      <c r="B9" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="5" t="s">
+      <c r="C9" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="5" t="s">
+      <c r="D9" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="5" t="s">
+      <c r="E9" s="4" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="4"/>
-      <c r="B10" s="6"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
+      <c r="A10" s="7"/>
+      <c r="B10" s="5"/>
+      <c r="C10" s="5"/>
+      <c r="D10" s="5"/>
+      <c r="E10" s="5"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="3">
+      <c r="A11" s="6">
         <v>5</v>
       </c>
-      <c r="B11" s="5" t="s">
+      <c r="B11" s="4" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="5" t="s">
+      <c r="C11" s="4" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="5" t="s">
+      <c r="D11" s="4" t="s">
         <v>24</v>
       </c>
-      <c r="E11" s="5" t="s">
+      <c r="E11" s="4" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="4"/>
-      <c r="B12" s="6"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
+      <c r="A12" s="7"/>
+      <c r="B12" s="5"/>
+      <c r="C12" s="5"/>
+      <c r="D12" s="5"/>
+      <c r="E12" s="5"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="2"/>
-      <c r="B13" s="2"/>
-      <c r="C13" s="2"/>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
+      <c r="A13" s="6">
+        <v>6</v>
+      </c>
+      <c r="B13" s="4" t="s">
+        <v>26</v>
+      </c>
+      <c r="C13" s="4" t="s">
+        <v>27</v>
+      </c>
+      <c r="D13" s="4" t="s">
+        <v>28</v>
+      </c>
+      <c r="E13" s="4" t="s">
+        <v>29</v>
+      </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="2"/>
-      <c r="B14" s="2"/>
-      <c r="C14" s="2"/>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
+      <c r="A14" s="7"/>
+      <c r="B14" s="5"/>
+      <c r="C14" s="5"/>
+      <c r="D14" s="5"/>
+      <c r="E14" s="5"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="2"/>
-      <c r="B15" s="2"/>
-      <c r="C15" s="2"/>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
+      <c r="A15" s="6"/>
+      <c r="B15" s="4"/>
+      <c r="C15" s="4"/>
+      <c r="D15" s="4"/>
+      <c r="E15" s="4"/>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
+      <c r="A16" s="7"/>
+      <c r="B16" s="5"/>
+      <c r="C16" s="5"/>
+      <c r="D16" s="5"/>
+      <c r="E16" s="5"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
@@ -765,33 +783,43 @@
       <c r="E18" s="2"/>
     </row>
   </sheetData>
-  <mergeCells count="26">
+  <mergeCells count="36">
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="E3:E4"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Septimo registro de decision
</commit_message>
<xml_diff>
--- a/Registro de decisiones.xlsx
+++ b/Registro de decisiones.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bdf77c9882a5fb43/Escritorio/laboratorio/novamarket-checkout-service/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="73" documentId="8_{F87E22D3-17D3-41A7-98E0-7C8DA0BE2010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CD5B3CDD-02AF-427A-A36C-AAF1B981B8EE}"/>
+  <xr:revisionPtr revIDLastSave="81" documentId="8_{F87E22D3-17D3-41A7-98E0-7C8DA0BE2010}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{87EA96CE-5F87-410A-8843-00EE25A107CA}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C6AF2156-5091-4E8F-AD24-4F68CDB55078}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="30" uniqueCount="30">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="34" uniqueCount="34">
   <si>
     <t>ID</t>
   </si>
@@ -129,6 +129,18 @@
   </si>
   <si>
     <t>No validar que cambios se realizó puede poner en riesgo el proyecto principal</t>
+  </si>
+  <si>
+    <t>Edición archivo instalacion en rama NM-103</t>
+  </si>
+  <si>
+    <t>Se creo una rama nueva de la principal en local para registrar el problema encontrado y validamos que no afecte otros servicios del proceso principal</t>
+  </si>
+  <si>
+    <t>Edición del archivo en la rama main</t>
+  </si>
+  <si>
+    <t>Puede generar otros problemas en cascada por realizar pequeñas ediciones en la rama principal</t>
   </si>
 </sst>
 </file>
@@ -226,7 +238,10 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
@@ -235,10 +250,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
   </cellXfs>
@@ -256,6 +268,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -585,13 +601,13 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A1" s="3" t="s">
+      <c r="A1" s="7" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="3"/>
-      <c r="C1" s="3"/>
-      <c r="D1" s="3"/>
-      <c r="E1" s="3"/>
+      <c r="B1" s="7"/>
+      <c r="C1" s="7"/>
+      <c r="D1" s="7"/>
+      <c r="E1" s="7"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
@@ -611,162 +627,172 @@
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A3" s="6">
+      <c r="A3" s="3">
         <v>1</v>
       </c>
-      <c r="B3" s="4" t="s">
+      <c r="B3" s="5" t="s">
         <v>6</v>
       </c>
-      <c r="C3" s="4" t="s">
+      <c r="C3" s="5" t="s">
         <v>7</v>
       </c>
-      <c r="D3" s="4" t="s">
+      <c r="D3" s="5" t="s">
         <v>8</v>
       </c>
-      <c r="E3" s="4" t="s">
+      <c r="E3" s="5" t="s">
         <v>9</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A4" s="7"/>
-      <c r="B4" s="5"/>
-      <c r="C4" s="5"/>
-      <c r="D4" s="5"/>
-      <c r="E4" s="5"/>
+      <c r="A4" s="4"/>
+      <c r="B4" s="6"/>
+      <c r="C4" s="6"/>
+      <c r="D4" s="6"/>
+      <c r="E4" s="6"/>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A5" s="6">
+      <c r="A5" s="3">
         <v>2</v>
       </c>
-      <c r="B5" s="4" t="s">
+      <c r="B5" s="5" t="s">
         <v>10</v>
       </c>
-      <c r="C5" s="4" t="s">
+      <c r="C5" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="D5" s="4" t="s">
+      <c r="D5" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="E5" s="4" t="s">
+      <c r="E5" s="5" t="s">
         <v>13</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A6" s="7"/>
-      <c r="B6" s="5"/>
-      <c r="C6" s="5"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
+      <c r="A6" s="4"/>
+      <c r="B6" s="6"/>
+      <c r="C6" s="6"/>
+      <c r="D6" s="6"/>
+      <c r="E6" s="6"/>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="6">
+      <c r="A7" s="3">
         <v>3</v>
       </c>
-      <c r="B7" s="4" t="s">
+      <c r="B7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C7" s="4" t="s">
+      <c r="C7" s="5" t="s">
         <v>15</v>
       </c>
-      <c r="D7" s="4" t="s">
+      <c r="D7" s="5" t="s">
         <v>16</v>
       </c>
-      <c r="E7" s="4" t="s">
+      <c r="E7" s="5" t="s">
         <v>17</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="7"/>
-      <c r="B8" s="5"/>
-      <c r="C8" s="5"/>
-      <c r="D8" s="5"/>
-      <c r="E8" s="5"/>
+      <c r="A8" s="4"/>
+      <c r="B8" s="6"/>
+      <c r="C8" s="6"/>
+      <c r="D8" s="6"/>
+      <c r="E8" s="6"/>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="6">
+      <c r="A9" s="3">
         <v>4</v>
       </c>
-      <c r="B9" s="4" t="s">
+      <c r="B9" s="5" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="4" t="s">
+      <c r="C9" s="5" t="s">
         <v>19</v>
       </c>
-      <c r="D9" s="4" t="s">
+      <c r="D9" s="5" t="s">
         <v>20</v>
       </c>
-      <c r="E9" s="4" t="s">
+      <c r="E9" s="5" t="s">
         <v>21</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A10" s="7"/>
-      <c r="B10" s="5"/>
-      <c r="C10" s="5"/>
-      <c r="D10" s="5"/>
-      <c r="E10" s="5"/>
+      <c r="A10" s="4"/>
+      <c r="B10" s="6"/>
+      <c r="C10" s="6"/>
+      <c r="D10" s="6"/>
+      <c r="E10" s="6"/>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A11" s="6">
+      <c r="A11" s="3">
         <v>5</v>
       </c>
-      <c r="B11" s="4" t="s">
+      <c r="B11" s="5" t="s">
         <v>22</v>
       </c>
-      <c r="C11" s="4" t="s">
+      <c r="C11" s="5" t="s">
         <v>23</v>
       </c>
-      <c r="D11" s="4" t="s">
+      <c r="D11" s="5" t="s">
         <v>24</v>
       </c>
-      <c r="E11" s="4" t="s">
+      <c r="E11" s="5" t="s">
         <v>25</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A12" s="7"/>
-      <c r="B12" s="5"/>
-      <c r="C12" s="5"/>
-      <c r="D12" s="5"/>
-      <c r="E12" s="5"/>
+      <c r="A12" s="4"/>
+      <c r="B12" s="6"/>
+      <c r="C12" s="6"/>
+      <c r="D12" s="6"/>
+      <c r="E12" s="6"/>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="6">
+      <c r="A13" s="3">
         <v>6</v>
       </c>
-      <c r="B13" s="4" t="s">
+      <c r="B13" s="5" t="s">
         <v>26</v>
       </c>
-      <c r="C13" s="4" t="s">
+      <c r="C13" s="5" t="s">
         <v>27</v>
       </c>
-      <c r="D13" s="4" t="s">
+      <c r="D13" s="5" t="s">
         <v>28</v>
       </c>
-      <c r="E13" s="4" t="s">
+      <c r="E13" s="5" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A14" s="7"/>
-      <c r="B14" s="5"/>
-      <c r="C14" s="5"/>
-      <c r="D14" s="5"/>
-      <c r="E14" s="5"/>
+      <c r="A14" s="4"/>
+      <c r="B14" s="6"/>
+      <c r="C14" s="6"/>
+      <c r="D14" s="6"/>
+      <c r="E14" s="6"/>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A15" s="6"/>
-      <c r="B15" s="4"/>
-      <c r="C15" s="4"/>
-      <c r="D15" s="4"/>
-      <c r="E15" s="4"/>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="7"/>
-      <c r="B16" s="5"/>
-      <c r="C16" s="5"/>
-      <c r="D16" s="5"/>
-      <c r="E16" s="5"/>
+      <c r="A15" s="3">
+        <v>7</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>30</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>31</v>
+      </c>
+      <c r="D15" s="5" t="s">
+        <v>32</v>
+      </c>
+      <c r="E15" s="5" t="s">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" ht="35.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A16" s="4"/>
+      <c r="B16" s="6"/>
+      <c r="C16" s="6"/>
+      <c r="D16" s="6"/>
+      <c r="E16" s="6"/>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="2"/>
@@ -784,42 +810,42 @@
     </row>
   </sheetData>
   <mergeCells count="36">
-    <mergeCell ref="A15:A16"/>
-    <mergeCell ref="B15:B16"/>
-    <mergeCell ref="C15:C16"/>
-    <mergeCell ref="D15:D16"/>
-    <mergeCell ref="E15:E16"/>
-    <mergeCell ref="A13:A14"/>
-    <mergeCell ref="B13:B14"/>
-    <mergeCell ref="C13:C14"/>
-    <mergeCell ref="D13:D14"/>
-    <mergeCell ref="E13:E14"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="B11:B12"/>
-    <mergeCell ref="C11:C12"/>
-    <mergeCell ref="D11:D12"/>
-    <mergeCell ref="E11:E12"/>
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="B9:B10"/>
-    <mergeCell ref="C9:C10"/>
-    <mergeCell ref="D9:D10"/>
-    <mergeCell ref="E9:E10"/>
-    <mergeCell ref="A7:A8"/>
-    <mergeCell ref="B7:B8"/>
-    <mergeCell ref="C7:C8"/>
-    <mergeCell ref="D7:D8"/>
-    <mergeCell ref="E7:E8"/>
-    <mergeCell ref="A5:A6"/>
-    <mergeCell ref="B5:B6"/>
-    <mergeCell ref="C5:C6"/>
-    <mergeCell ref="D5:D6"/>
-    <mergeCell ref="E5:E6"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="C3:C4"/>
     <mergeCell ref="A3:A4"/>
     <mergeCell ref="B3:B4"/>
     <mergeCell ref="D3:D4"/>
     <mergeCell ref="E3:E4"/>
+    <mergeCell ref="A5:A6"/>
+    <mergeCell ref="B5:B6"/>
+    <mergeCell ref="C5:C6"/>
+    <mergeCell ref="D5:D6"/>
+    <mergeCell ref="E5:E6"/>
+    <mergeCell ref="A7:A8"/>
+    <mergeCell ref="B7:B8"/>
+    <mergeCell ref="C7:C8"/>
+    <mergeCell ref="D7:D8"/>
+    <mergeCell ref="E7:E8"/>
+    <mergeCell ref="A9:A10"/>
+    <mergeCell ref="B9:B10"/>
+    <mergeCell ref="C9:C10"/>
+    <mergeCell ref="D9:D10"/>
+    <mergeCell ref="E9:E10"/>
+    <mergeCell ref="A11:A12"/>
+    <mergeCell ref="B11:B12"/>
+    <mergeCell ref="C11:C12"/>
+    <mergeCell ref="D11:D12"/>
+    <mergeCell ref="E11:E12"/>
+    <mergeCell ref="A13:A14"/>
+    <mergeCell ref="B13:B14"/>
+    <mergeCell ref="C13:C14"/>
+    <mergeCell ref="D13:D14"/>
+    <mergeCell ref="E13:E14"/>
+    <mergeCell ref="A15:A16"/>
+    <mergeCell ref="B15:B16"/>
+    <mergeCell ref="C15:C16"/>
+    <mergeCell ref="D15:D16"/>
+    <mergeCell ref="E15:E16"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>